<commit_message>
passage des competences valide en vert
</commit_message>
<xml_diff>
--- a/documents/Tableau-synthese-E4.xlsx
+++ b/documents/Tableau-synthese-E4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://efrei365net-my.sharepoint.com/personal/noham_tayaa_efrei_net/Documents/BTS-SIO/BTS-2/E5 - Support et mise a disposition des services informatique/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://efrei365net-my.sharepoint.com/personal/noham_tayaa_efrei_net/Documents/BTS-SIO/Portfolio/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="11_BDF6366FA7694CE96F0AED02F7301D2C05FF6A3B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A38B6A84-CC60-4860-B396-CADEF1A3DD6B}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="11_BDF6366FA7694CE96F0AED02F7301D2C05FF6A3B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA0EA7EC-CC9C-44B3-BB69-91AB91B341B7}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="0" windowWidth="15588" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
@@ -227,12 +227,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="29">
@@ -626,7 +632,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -688,9 +694,51 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -715,47 +763,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1076,56 +1088,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="21"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="28" t="s">
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="23"/>
-      <c r="H3" s="29"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="43"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="27"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1137,22 +1149,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="40" t="s">
+      <c r="A5" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="41"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="35"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="31" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1175,8 +1187,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="31"/>
-      <c r="B7" s="39"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1232,16 +1244,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="27"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1283,7 +1295,7 @@
         <v>27</v>
       </c>
       <c r="B9" s="10"/>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="44" t="s">
         <v>25</v>
       </c>
       <c r="D9" s="16"/>
@@ -1336,7 +1348,7 @@
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
-      <c r="G10" s="16" t="s">
+      <c r="G10" s="44" t="s">
         <v>25</v>
       </c>
       <c r="H10" s="17"/>
@@ -1382,7 +1394,7 @@
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="16"/>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="44" t="s">
         <v>25</v>
       </c>
       <c r="E11" s="16"/>
@@ -1434,10 +1446,10 @@
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
-      <c r="G12" s="16" t="s">
+      <c r="G12" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="H12" s="17" t="s">
+      <c r="H12" s="45" t="s">
         <v>25</v>
       </c>
       <c r="I12"/>
@@ -1747,16 +1759,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="35" t="s">
+      <c r="A19" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="36"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="37"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="30"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1802,7 +1814,7 @@
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
-      <c r="G20" s="16" t="s">
+      <c r="G20" s="44" t="s">
         <v>25</v>
       </c>
       <c r="H20" s="17"/>
@@ -1843,15 +1855,15 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="21" t="s">
         <v>33</v>
       </c>
       <c r="B21" s="10"/>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="44" t="s">
         <v>25</v>
       </c>
       <c r="D21" s="16"/>
-      <c r="E21" s="16" t="s">
+      <c r="E21" s="44" t="s">
         <v>25</v>
       </c>
       <c r="F21" s="16"/>
@@ -1899,7 +1911,7 @@
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="16"/>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="44" t="s">
         <v>25</v>
       </c>
       <c r="E22" s="16"/>
@@ -2123,16 +2135,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A27" s="35" t="s">
+      <c r="A27" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="36"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="36"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="37"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="30"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2178,7 +2190,7 @@
       <c r="D28" s="16"/>
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
-      <c r="G28" s="16" t="s">
+      <c r="G28" s="44" t="s">
         <v>25</v>
       </c>
       <c r="H28" s="17"/>
@@ -2226,7 +2238,7 @@
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
-      <c r="F29" s="16" t="s">
+      <c r="F29" s="44" t="s">
         <v>25</v>
       </c>
       <c r="G29" s="16"/>
@@ -2272,7 +2284,7 @@
         <v>33</v>
       </c>
       <c r="B30" s="10"/>
-      <c r="C30" s="16" t="s">
+      <c r="C30" s="44" t="s">
         <v>25</v>
       </c>
       <c r="D30" s="16"/>
@@ -2589,6 +2601,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2596,11 +2613,6 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>